<commit_message>
Sep 22 refresh: presentation fixes — city normalization, Account List cities, Territory kept-by-cell, short-day flags, doc wording
- City labels normalized (St/Saint, Clarkston village variants, Twp) and
  blank MMC cities parsed from the address or peers' zip; Account List and
  By City now agree; no 'Nan'/'Michigan' labels anywhere.
- Territory 'Kept (W9)' counted by the account's home cell; Weekly Plan W9
  notes carry the own-and-neighbouring qualifier; days under 8 stops are
  flagged SHORT DAY with the finish-early instruction.
- Parking-lot geography paragraph attributes wide days correctly; pocket
  counts show only untouched prospects; glossary cell count and the
  duplicated §5 banner fixed; docs regenerated from the artifacts.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
+++ b/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
@@ -1954,7 +1954,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>transition — 6 Sep 3 W9 producer stops kept (built from J-R03)</t>
+          <t>transition — 6 Sep 3 W9 producer stops kept on this day (own and neighbouring Sep 3 days; built from J-R03)</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>transition — 7 Sep 3 W9 producer stops kept (built from J-R04)</t>
+          <t>transition — 7 Sep 3 W9 producer stops kept on this day (own and neighbouring Sep 3 days; built from J-R04)</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>transition — 5 Sep 3 W9 producer stops kept (built from J-R06)</t>
+          <t>transition — 5 Sep 3 W9 producer stops kept on this day (own and neighbouring Sep 3 days; built from J-R06)</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>transition — 2 Sep 3 W9 producer stops kept (built from J-R07)</t>
+          <t>transition — 2 Sep 3 W9 producer stops kept on this day (own and neighbouring Sep 3 days; built from J-R07)</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>transition — 2 Sep 3 W9 producer stops kept (built from J-R10)</t>
+          <t>transition — 2 Sep 3 W9 producer stops kept on this day (own and neighbouring Sep 3 days; built from J-R10)</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
@@ -37240,7 +37240,7 @@
       </c>
       <c r="K563" s="3" t="inlineStr">
         <is>
-          <t>Brownstown Twp</t>
+          <t>Brownstown Township</t>
         </is>
       </c>
       <c r="L563" s="4" t="inlineStr">
@@ -38021,7 +38021,7 @@
         <v>2</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3" s="6" t="n"/>
       <c r="I3" s="7" t="inlineStr">
@@ -38159,7 +38159,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="7" t="inlineStr">
@@ -38195,7 +38195,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H8" s="6" t="n"/>
       <c r="I8" s="7" t="inlineStr">
@@ -38231,7 +38231,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" s="6" t="n"/>
       <c r="I9" s="7" t="inlineStr">
@@ -38266,7 +38266,9 @@
       <c r="F10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="6" t="n"/>
+      <c r="G10" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="7" t="inlineStr">
         <is>
@@ -38301,7 +38303,7 @@
         <v>7</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="7" t="inlineStr">
@@ -49246,7 +49248,7 @@
       </c>
       <c r="J180" s="6" t="inlineStr">
         <is>
-          <t>Nan</t>
+          <t>Canton</t>
         </is>
       </c>
       <c r="K180" s="7" t="inlineStr">
@@ -52947,7 +52949,7 @@
       </c>
       <c r="J243" s="6" t="inlineStr">
         <is>
-          <t>Brownstown</t>
+          <t>Brownstown Township</t>
         </is>
       </c>
       <c r="K243" s="7" t="inlineStr">
@@ -57428,7 +57430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -57569,7 +57571,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>8</v>
@@ -57581,7 +57583,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>15</v>
@@ -58456,7 +58458,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Brownstown Twp</t>
+          <t>Brownstown Township</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -58522,7 +58524,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Rd</t>
+          <t>Northville</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -58548,21 +58550,21 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>J-A09</t>
+          <t>J-A01</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Northville</t>
+          <t>Walled Lake</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="6" t="n">
         <v>0</v>
@@ -58571,10 +58573,10 @@
         <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>0</v>
@@ -58588,18 +58590,18 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Walled Lake</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="E36" s="6" t="n">
         <v>0</v>
       </c>
@@ -58607,21 +58609,21 @@
         <v>0</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>J-A01</t>
+          <t>J-A03</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Sterling Heights</t>
+          <t>Howell</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
@@ -58631,11 +58633,11 @@
         <v>0</v>
       </c>
       <c r="D37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
       </c>
@@ -58646,39 +58648,6 @@
         <v>0</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>J-A03</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Howell</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>J-A01</t>
         </is>

</xml_diff>

<commit_message>
Oct 9 refresh: stranded-Tier-1 pass, recap reframed by day list, app check-in markers for W9/W10
- Scheduler runs two passes: cell sequence ranked freely, then overdue Tier 1s whose cells earn no day are pulled onto the nearest day (≤12 mi), displacing a prospect first — 19 placed; overdue Tier 1 first week W11 83 · W12 31 · W13 12 · W14 4
- Recap keyed by day lists with totals, planned-stop credit counts any PL's check-in, ledger 'last visit before the week' only
- App W9/W10 stops show ✔ visited / not visited; relationship workbook note updated to Oct 9 visit-days; parking-lot and v14 banner regenerated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
+++ b/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
@@ -2429,7 +2429,7 @@
         <v>10</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0</v>
@@ -2438,17 +2438,17 @@
         <v>0</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Livonia (2) • Garden City (2)</t>
+          <t>Dearborn (3) • Livonia (2)</t>
         </is>
       </c>
       <c r="J44" s="4" t="n"/>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=20001%20West%20Seven%20Mile%20Road%2C%20Detroit%2C%20Michigan%2C%2048219&amp;waypoints=20290%20Middlebelt%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C28701%20Plymouth%20Rd%2C%20Livonia%2C%20Michigan%2C%2048150%7C5823%20MIDDLEBELT%20RD%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C29454%20Ford%20Road%2C%20Garden%20City%2C%20Michigan%2C%2048135%7C27155%20CHERRY%20HILL%20RD%2C%20INKSTER%2C%20MI%2C%2048141%7C23870%20Michigan%20Ave%2C%20Dearborn%2C%20MI%20nan%7C21801%20GODDARD%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C22361%20W%20VILLAGE%20DR%20STE%20102%2C%20DEARBORN%2C%20MI%2C%2048124%7C16226%20Grand%20River%20Ave%2C%20Detroit%2C%20Michigan%2C%2048227</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=20001%20West%20Seven%20Mile%20Road%2C%20Detroit%2C%20Michigan%2C%2048219&amp;waypoints=20290%20Middlebelt%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C28701%20Plymouth%20Rd%2C%20Livonia%2C%20Michigan%2C%2048150%7C5823%20MIDDLEBELT%20RD%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C29454%20Ford%20Road%2C%20Garden%20City%2C%20Michigan%2C%2048135%7C27155%20CHERRY%20HILL%20RD%2C%20INKSTER%2C%20MI%2C%2048141%7C23870%20Michigan%20Ave%2C%20Dearborn%2C%20MI%20nan%7C22361%20W%20VILLAGE%20DR%20STE%20102%2C%20DEARBORN%2C%20MI%2C%2048124%7C17000%20Hubbard%20Dr%2C%20Dearborn%2C%20Michigan%2C%2048126%7C16226%20Grand%20River%20Ave%2C%20Detroit%2C%20Michigan%2C%2048227</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
         <v>10</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>8</v>
@@ -2782,17 +2782,17 @@
         <v>0</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Dearborn (3) • Livonia (2)</t>
+          <t>Livonia (2) • Dearborn Heights (2)</t>
         </is>
       </c>
       <c r="J52" s="4" t="n"/>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=13244%20W%20Warren%20Ave%2C%20Dearborn%2C%20Michigan%2C%2048126&amp;waypoints=14555%20Levan%20Rd%20suite%20308%2C%20Livonia%2C%20Michigan%2C%2048154%7C28479%207%20MILE%20RD%2C%20LIVONIA%2C%20MI%2C%2048152%7C25350%20West%20Warren%20Street%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048127%7C29150%20FORD%20RD%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C27250%20Cherry%20Hill%20Road%2C%20Dearborn%20Heights%2C%20MI%2048127%7C4020%20Venoy%20Rd%20suite%20400%2C%20Wayne%2C%20Michigan%2C%2048184%7C15100%20S%20PLAZA%20DR%2C%20TAYLOR%2C%20MI%2C%2048180%7C17000%20Hubbard%20Dr%2C%20Dearborn%2C%20Michigan%2C%2048126%7C5245%20Schaefer%20Rd%2C%20Dearborn%2C%20Michigan%2C%2048126</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=13244%20W%20Warren%20Ave%2C%20Dearborn%2C%20Michigan%2C%2048126&amp;waypoints=14555%20Levan%20Rd%20suite%20308%2C%20Livonia%2C%20Michigan%2C%2048154%7C28479%207%20MILE%20RD%2C%20LIVONIA%2C%20MI%2C%2048152%7C25350%20West%20Warren%20Street%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048127%7C29150%20FORD%20RD%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C27250%20Cherry%20Hill%20Road%2C%20Dearborn%20Heights%2C%20MI%2048127%7C4020%20Venoy%20Rd%20suite%20400%2C%20Wayne%2C%20Michigan%2C%2048184%7C15100%20S%20PLAZA%20DR%2C%20TAYLOR%2C%20MI%2C%2048180%7C21801%20GODDARD%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C5245%20Schaefer%20Rd%2C%20Dearborn%2C%20Michigan%2C%2048126</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
         <v>10</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>0</v>
@@ -2997,17 +2997,17 @@
         <v>0</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Dearborn (3) • Taylor (3)</t>
+          <t>Dearborn (4) • Taylor (2)</t>
         </is>
       </c>
       <c r="J57" s="4" t="n"/>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2865%20West%20Road%2C%20Trenton%2C%20Michigan%2C%2048183&amp;waypoints=3133%20South%20Telegraph%20Road%2C%20Dearborn%2C%20Michigan%2C%2048124%7C22361%20W%20VILLAGE%20DR%20STE%20102%2C%20DEARBORN%2C%20MI%2C%2048124%7C3815%20Pelham%20Street%2C%20Dearborn%2C%20Michigan%2C%2048124%7C9340%20TELEGRAPH%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C12701%20Telegraph%20Rd%2C%20ste%20103%2C%20TAYLOR%2C%20Michigan%2C%2048180%7C11368%20Allen%20Road%2C%20Taylor%2C%20Michigan%2C%2048180%7C15450%20Northline%20Road%2C%20Southgate%2C%20MI%2048195%7C2300%20Biddle%20Avenue%2C%20Wyandotte%2C%20Michigan%2C%2048192%7C13909%20Pennsylvania%20Road%2C%20Suite%20B%2C%20Riverview%2C%20Michigan%2C%2048193</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2865%20West%20Road%2C%20Trenton%2C%20Michigan%2C%2048183&amp;waypoints=3133%20South%20Telegraph%20Road%2C%20Dearborn%2C%20Michigan%2C%2048124%7C22361%20W%20VILLAGE%20DR%20STE%20102%2C%20DEARBORN%2C%20MI%2C%2048124%7C17000%20Hubbard%20Dr%2C%20Dearborn%2C%20Michigan%2C%2048126%7C3815%20Pelham%20Street%2C%20Dearborn%2C%20Michigan%2C%2048124%7C9340%20TELEGRAPH%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C11368%20Allen%20Road%2C%20Taylor%2C%20Michigan%2C%2048180%7C15450%20Northline%20Road%2C%20Southgate%2C%20MI%2048195%7C2300%20Biddle%20Avenue%2C%20Wyandotte%2C%20Michigan%2C%2048192%7C13909%20Pennsylvania%20Road%2C%20Suite%20B%2C%20Riverview%2C%20Michigan%2C%2048193</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
         <v>10</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>3</v>
@@ -3083,17 +3083,17 @@
         <v>1</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Southgate (2) • Southfield (2)</t>
+          <t>Taylor (2) • Southgate (2)</t>
         </is>
       </c>
       <c r="J59" s="4" t="n"/>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=27207%20Lahser%20Rd%2C%20Southfield%2C%20Michigan%2C%2048034&amp;waypoints=36475%205%20MILE%20RD%2C%20LIVONIA%2C%20Michigan%2C%2048154%7C34659%20West%20Michigan%20Avenue%2C%20Wayne%2C%20Michigan%2C%2048184%7C25500%20GODDARD%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C19727%20Allen%20Rd%2C%20Ste%2011%2C%20Brownstown%20Twp%2C%20Michigan%2C%2048183%7C13636%20Dix%20Toledo%2C%20Southgate%2C%20MI%2C%20481952432%7C15555%20Northline%20Road%2C%20Southgate%2C%20Michigan%2C%2048195%7C3902%20Monroe%20St%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048125%7C17000%20Hubbard%20Dr%2C%20Dearborn%2C%20Michigan%2C%2048126%7C22250%20Providence%20Drive%2C%20ste%20401%2C%20Southfield%2C%20Michigan%2C%2048075</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=27207%20Lahser%20Rd%2C%20Southfield%2C%20Michigan%2C%2048034&amp;waypoints=36475%205%20MILE%20RD%2C%20LIVONIA%2C%20Michigan%2C%2048154%7C34659%20West%20Michigan%20Avenue%2C%20Wayne%2C%20Michigan%2C%2048184%7C25500%20GODDARD%20RD%2C%20TAYLOR%2C%20MI%2C%2048180%7C12701%20Telegraph%20Rd%2C%20ste%20103%2C%20TAYLOR%2C%20Michigan%2C%2048180%7C19727%20Allen%20Rd%2C%20Ste%2011%2C%20Brownstown%20Twp%2C%20Michigan%2C%2048183%7C13636%20Dix%20Toledo%2C%20Southgate%2C%20MI%2C%20481952432%7C15555%20Northline%20Road%2C%20Southgate%2C%20Michigan%2C%2048195%7C3902%20Monroe%20St%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048125%7C22250%20Providence%20Drive%2C%20ste%20401%2C%20Southfield%2C%20Michigan%2C%2048075</t>
         </is>
       </c>
     </row>
@@ -27321,22 +27321,22 @@
       </c>
       <c r="D391" s="4" t="inlineStr">
         <is>
-          <t>📝 DOWNRIVER INTERNISTS, PC</t>
+          <t>📝 TENNY INTERNAL MEDICINE, PLLC</t>
         </is>
       </c>
       <c r="E391" s="4" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Mar 5</t>
+          <t>Tier 1 producer · last check-in Sep 24</t>
         </is>
       </c>
       <c r="F391" s="3" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G391" s="3" t="inlineStr">
         <is>
-          <t>0889eef0-5cc1-4032-b658-e4a9c719c997</t>
+          <t>3effe9bc-8576-4eee-ba7e-9bf99eb7d1fa</t>
         </is>
       </c>
       <c r="H391" s="3" t="inlineStr">
@@ -27350,16 +27350,16 @@
         </is>
       </c>
       <c r="J391" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K391" s="3" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>Dearborn</t>
         </is>
       </c>
       <c r="L391" s="4" t="inlineStr">
         <is>
-          <t>21801 GODDARD RD, TAYLOR, MI, 48180</t>
+          <t>22361 W VILLAGE DR STE 102, DEARBORN, MI, 48124</t>
         </is>
       </c>
       <c r="M391" s="4" t="n"/>
@@ -27381,12 +27381,12 @@
       </c>
       <c r="D392" s="4" t="inlineStr">
         <is>
-          <t>📝 TENNY INTERNAL MEDICINE, PLLC</t>
+          <t>📝 COREWELL HEALTH  INTERNAL MEDICINE DEARBORN</t>
         </is>
       </c>
       <c r="E392" s="4" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 24</t>
+          <t>Tier 1 producer · last check-in Aug 26</t>
         </is>
       </c>
       <c r="F392" s="3" t="inlineStr">
@@ -27396,7 +27396,7 @@
       </c>
       <c r="G392" s="3" t="inlineStr">
         <is>
-          <t>3effe9bc-8576-4eee-ba7e-9bf99eb7d1fa</t>
+          <t>9d286e7b-6017-417c-8a6b-763fe942c9c2</t>
         </is>
       </c>
       <c r="H392" s="3" t="inlineStr">
@@ -27419,7 +27419,7 @@
       </c>
       <c r="L392" s="4" t="inlineStr">
         <is>
-          <t>22361 W VILLAGE DR STE 102, DEARBORN, MI, 48124</t>
+          <t>17000 Hubbard Dr, Dearborn, Michigan, 48126</t>
         </is>
       </c>
       <c r="M392" s="4" t="n"/>
@@ -32181,22 +32181,22 @@
       </c>
       <c r="D472" s="4" t="inlineStr">
         <is>
-          <t>📝 COREWELL HEALTH  INTERNAL MEDICINE DEARBORN</t>
+          <t>📝 DOWNRIVER INTERNISTS, PC</t>
         </is>
       </c>
       <c r="E472" s="4" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 26</t>
+          <t>Prospect · last check-in Mar 5</t>
         </is>
       </c>
       <c r="F472" s="3" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G472" s="3" t="inlineStr">
         <is>
-          <t>9d286e7b-6017-417c-8a6b-763fe942c9c2</t>
+          <t>0889eef0-5cc1-4032-b658-e4a9c719c997</t>
         </is>
       </c>
       <c r="H472" s="3" t="inlineStr">
@@ -32210,16 +32210,16 @@
         </is>
       </c>
       <c r="J472" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K472" s="3" t="inlineStr">
         <is>
-          <t>Dearborn</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="L472" s="4" t="inlineStr">
         <is>
-          <t>17000 Hubbard Dr, Dearborn, Michigan, 48126</t>
+          <t>21801 GODDARD RD, TAYLOR, MI, 48180</t>
         </is>
       </c>
       <c r="M472" s="4" t="n"/>
@@ -34881,12 +34881,12 @@
       </c>
       <c r="D517" s="4" t="inlineStr">
         <is>
-          <t>📝 PelHam Primary Care</t>
+          <t>📝 COREWELL HEALTH  INTERNAL MEDICINE DEARBORN</t>
         </is>
       </c>
       <c r="E517" s="4" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 23</t>
+          <t>Tier 1 producer · last check-in Aug 26</t>
         </is>
       </c>
       <c r="F517" s="3" t="inlineStr">
@@ -34896,7 +34896,7 @@
       </c>
       <c r="G517" s="3" t="inlineStr">
         <is>
-          <t>d4c2e8cb-a4bb-454f-bc5c-8425cff6d293</t>
+          <t>9d286e7b-6017-417c-8a6b-763fe942c9c2</t>
         </is>
       </c>
       <c r="H517" s="3" t="inlineStr">
@@ -34919,7 +34919,7 @@
       </c>
       <c r="L517" s="4" t="inlineStr">
         <is>
-          <t>3815 Pelham Street, Dearborn, Michigan, 48124</t>
+          <t>17000 Hubbard Dr, Dearborn, Michigan, 48126</t>
         </is>
       </c>
       <c r="M517" s="4" t="n"/>
@@ -34941,22 +34941,22 @@
       </c>
       <c r="D518" s="4" t="inlineStr">
         <is>
-          <t>📝 BEAUMONT FAMILY MEDICINE CLINIC TAYLOR</t>
+          <t>📝 PelHam Primary Care</t>
         </is>
       </c>
       <c r="E518" s="4" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Apr 8</t>
+          <t>Tier 1 producer · last check-in Sep 23</t>
         </is>
       </c>
       <c r="F518" s="3" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G518" s="3" t="inlineStr">
         <is>
-          <t>ca75c2bf-f7ff-43df-9399-5f78f3147237</t>
+          <t>d4c2e8cb-a4bb-454f-bc5c-8425cff6d293</t>
         </is>
       </c>
       <c r="H518" s="3" t="inlineStr">
@@ -34970,16 +34970,16 @@
         </is>
       </c>
       <c r="J518" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K518" s="3" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>Dearborn</t>
         </is>
       </c>
       <c r="L518" s="4" t="inlineStr">
         <is>
-          <t>9340 TELEGRAPH RD, TAYLOR, MI, 48180</t>
+          <t>3815 Pelham Street, Dearborn, Michigan, 48124</t>
         </is>
       </c>
       <c r="M518" s="4" t="n"/>
@@ -35001,7 +35001,7 @@
       </c>
       <c r="D519" s="4" t="inlineStr">
         <is>
-          <t>📝 PARK PLACE FAMILY PRACTICE AND INTERNAL MEDICINE</t>
+          <t>📝 BEAUMONT FAMILY MEDICINE CLINIC TAYLOR</t>
         </is>
       </c>
       <c r="E519" s="4" t="inlineStr">
@@ -35016,12 +35016,12 @@
       </c>
       <c r="G519" s="3" t="inlineStr">
         <is>
-          <t>f8f13fd9-1135-4385-b6ba-7542d202b63a</t>
+          <t>ca75c2bf-f7ff-43df-9399-5f78f3147237</t>
         </is>
       </c>
       <c r="H519" s="3" t="inlineStr">
         <is>
-          <t>Pain</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I519" s="3" t="inlineStr">
@@ -35039,7 +35039,7 @@
       </c>
       <c r="L519" s="4" t="inlineStr">
         <is>
-          <t>12701 Telegraph Rd, ste 103, TAYLOR, Michigan, 48180</t>
+          <t>9340 TELEGRAPH RD, TAYLOR, MI, 48180</t>
         </is>
       </c>
       <c r="M519" s="4" t="n"/>
@@ -36141,12 +36141,12 @@
       </c>
       <c r="D538" s="4" t="inlineStr">
         <is>
-          <t>📝 AMINI HEALTHCARE, PLLC</t>
+          <t>📝 PARK PLACE FAMILY PRACTICE AND INTERNAL MEDICINE</t>
         </is>
       </c>
       <c r="E538" s="4" t="inlineStr">
         <is>
-          <t>Prospect · last check-in May 29</t>
+          <t>Prospect · last check-in Apr 8</t>
         </is>
       </c>
       <c r="F538" s="3" t="inlineStr">
@@ -36156,12 +36156,12 @@
       </c>
       <c r="G538" s="3" t="inlineStr">
         <is>
-          <t>51be485c-bce1-4997-8e82-1463313f4617</t>
+          <t>f8f13fd9-1135-4385-b6ba-7542d202b63a</t>
         </is>
       </c>
       <c r="H538" s="3" t="inlineStr">
         <is>
-          <t>Orthopedic</t>
+          <t>Pain</t>
         </is>
       </c>
       <c r="I538" s="3" t="inlineStr">
@@ -36174,12 +36174,12 @@
       </c>
       <c r="K538" s="3" t="inlineStr">
         <is>
-          <t>Brownstown Township</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="L538" s="4" t="inlineStr">
         <is>
-          <t>19727 Allen Rd, Ste 11, Brownstown Twp, Michigan, 48183</t>
+          <t>12701 Telegraph Rd, ste 103, TAYLOR, Michigan, 48180</t>
         </is>
       </c>
       <c r="M538" s="4" t="n"/>
@@ -36201,27 +36201,27 @@
       </c>
       <c r="D539" s="4" t="inlineStr">
         <is>
-          <t>📝 City Medical - Southgate</t>
+          <t>📝 AMINI HEALTHCARE, PLLC</t>
         </is>
       </c>
       <c r="E539" s="4" t="inlineStr">
         <is>
-          <t>Tier 2 ortho · last check-in Sep 21</t>
+          <t>Prospect · last check-in May 29</t>
         </is>
       </c>
       <c r="F539" s="3" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G539" s="3" t="inlineStr">
         <is>
-          <t>1326021262</t>
+          <t>51be485c-bce1-4997-8e82-1463313f4617</t>
         </is>
       </c>
       <c r="H539" s="3" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Orthopedic</t>
         </is>
       </c>
       <c r="I539" s="3" t="inlineStr">
@@ -36234,12 +36234,12 @@
       </c>
       <c r="K539" s="3" t="inlineStr">
         <is>
-          <t>Southgate</t>
+          <t>Brownstown Township</t>
         </is>
       </c>
       <c r="L539" s="4" t="inlineStr">
         <is>
-          <t>13636 Dix Toledo, Southgate, MI, 481952432</t>
+          <t>19727 Allen Rd, Ste 11, Brownstown Twp, Michigan, 48183</t>
         </is>
       </c>
       <c r="M539" s="4" t="n"/>
@@ -36261,7 +36261,7 @@
       </c>
       <c r="D540" s="4" t="inlineStr">
         <is>
-          <t>📝 PEDIATRIC AND ADOLESCENT CENTER</t>
+          <t>📝 City Medical - Southgate</t>
         </is>
       </c>
       <c r="E540" s="4" t="inlineStr">
@@ -36276,12 +36276,12 @@
       </c>
       <c r="G540" s="3" t="inlineStr">
         <is>
-          <t>31fe13d8-1060-4c98-bf75-61f09e803121</t>
+          <t>1326021262</t>
         </is>
       </c>
       <c r="H540" s="3" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I540" s="3" t="inlineStr">
@@ -36299,7 +36299,7 @@
       </c>
       <c r="L540" s="4" t="inlineStr">
         <is>
-          <t>15555 Northline Road, Southgate, Michigan, 48195</t>
+          <t>13636 Dix Toledo, Southgate, MI, 481952432</t>
         </is>
       </c>
       <c r="M540" s="4" t="n"/>
@@ -36321,27 +36321,27 @@
       </c>
       <c r="D541" s="4" t="inlineStr">
         <is>
-          <t>📝 Primary Care Center</t>
+          <t>📝 PEDIATRIC AND ADOLESCENT CENTER</t>
         </is>
       </c>
       <c r="E541" s="4" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Jun 17</t>
+          <t>Tier 2 ortho · last check-in Sep 21</t>
         </is>
       </c>
       <c r="F541" s="3" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="G541" s="3" t="inlineStr">
         <is>
-          <t>814ed74d-d989-4209-bc8c-83f8248094b6</t>
+          <t>31fe13d8-1060-4c98-bf75-61f09e803121</t>
         </is>
       </c>
       <c r="H541" s="3" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I541" s="3" t="inlineStr">
@@ -36354,12 +36354,12 @@
       </c>
       <c r="K541" s="3" t="inlineStr">
         <is>
-          <t>Dearborn Heights</t>
+          <t>Southgate</t>
         </is>
       </c>
       <c r="L541" s="4" t="inlineStr">
         <is>
-          <t>3902 Monroe St, Dearborn Heights, Michigan, 48125</t>
+          <t>15555 Northline Road, Southgate, Michigan, 48195</t>
         </is>
       </c>
       <c r="M541" s="4" t="n"/>
@@ -36381,22 +36381,22 @@
       </c>
       <c r="D542" s="4" t="inlineStr">
         <is>
-          <t>📝 COREWELL HEALTH  INTERNAL MEDICINE DEARBORN</t>
+          <t>📝 Primary Care Center</t>
         </is>
       </c>
       <c r="E542" s="4" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 26</t>
+          <t>Prospect · last check-in Jun 17</t>
         </is>
       </c>
       <c r="F542" s="3" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G542" s="3" t="inlineStr">
         <is>
-          <t>9d286e7b-6017-417c-8a6b-763fe942c9c2</t>
+          <t>814ed74d-d989-4209-bc8c-83f8248094b6</t>
         </is>
       </c>
       <c r="H542" s="3" t="inlineStr">
@@ -36410,16 +36410,16 @@
         </is>
       </c>
       <c r="J542" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K542" s="3" t="inlineStr">
         <is>
-          <t>Dearborn</t>
+          <t>Dearborn Heights</t>
         </is>
       </c>
       <c r="L542" s="4" t="inlineStr">
         <is>
-          <t>17000 Hubbard Dr, Dearborn, Michigan, 48126</t>
+          <t>3902 Monroe St, Dearborn Heights, Michigan, 48125</t>
         </is>
       </c>
       <c r="M542" s="4" t="n"/>
@@ -65206,7 +65206,7 @@
         <v>50</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>10</v>
@@ -65215,7 +65215,7 @@
         <v>3</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -65231,7 +65231,7 @@
         <v>50</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>22</v>
@@ -65240,7 +65240,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -65256,7 +65256,7 @@
         <v>50</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>7</v>
@@ -65265,7 +65265,7 @@
         <v>2</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -65281,7 +65281,7 @@
         <v>47</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>23</v>
@@ -65290,7 +65290,7 @@
         <v>3</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">

</xml_diff>